<commit_message>
correccion de errores en importacion de actividades, y opcion de exportar consolidado de actividades
</commit_message>
<xml_diff>
--- a/assets/templates/plantilla_importacion_actividad.xlsx
+++ b/assets/templates/plantilla_importacion_actividad.xlsx
@@ -798,7 +798,7 @@
       <c r="S2" s="14" t="n"/>
       <c r="T2" s="15" t="n"/>
     </row>
-    <row r="3">
+    <row r="3" ht="36" customHeight="1">
       <c r="A3" s="16" t="inlineStr">
         <is>
           <t>FECHA</t>
@@ -836,7 +836,7 @@
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>COMITES DE SALUD</t>
+          <t>CANTIDAD DE COMITÉS DE SALUD (0-99)</t>
         </is>
       </c>
       <c r="I3" s="16" t="inlineStr">

</xml_diff>

<commit_message>
mejoras para la seleccion filtrada de parroquias y asic segun el municipio
</commit_message>
<xml_diff>
--- a/assets/templates/plantilla_importacion_actividad.xlsx
+++ b/assets/templates/plantilla_importacion_actividad.xlsx
@@ -8,16 +8,51 @@
   </bookViews>
   <sheets>
     <sheet name="Actividades" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Catalogos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="CatalogoActividades">'Catalogos'!$A$2:$A$9</definedName>
+    <definedName name="CatalogoASIC">'Catalogos'!$B$2:$B$26</definedName>
+    <definedName name="CatalogoMunicipios">'Catalogos'!$C$2:$C$30</definedName>
+    <definedName name="Parroquia1">'Catalogos'!$D$2:$D$2</definedName>
+    <definedName name="Parroquia2">'Catalogos'!$E$2:$E$2</definedName>
+    <definedName name="Parroquia3">'Catalogos'!$F$2:$F$4</definedName>
+    <definedName name="Parroquia4">'Catalogos'!$G$2:$G$5</definedName>
+    <definedName name="Parroquia5">'Catalogos'!$H$2:$H$4</definedName>
+    <definedName name="Parroquia6">'Catalogos'!$I$2:$I$2</definedName>
+    <definedName name="Parroquia7">'Catalogos'!$J$2:$J$4</definedName>
+    <definedName name="Parroquia8">'Catalogos'!$K$2:$K$2</definedName>
+    <definedName name="Parroquia9">'Catalogos'!$L$2:$L$4</definedName>
+    <definedName name="Parroquia10">'Catalogos'!$M$2:$M$2</definedName>
+    <definedName name="Parroquia11">'Catalogos'!$N$2:$N$4</definedName>
+    <definedName name="Parroquia12">'Catalogos'!$O$2:$O$2</definedName>
+    <definedName name="Parroquia13">'Catalogos'!$P$2:$P$5</definedName>
+    <definedName name="Parroquia14">'Catalogos'!$Q$2:$Q$4</definedName>
+    <definedName name="Parroquia15">'Catalogos'!$R$2:$R$4</definedName>
+    <definedName name="Parroquia16">'Catalogos'!$S$2:$S$5</definedName>
+    <definedName name="Parroquia17">'Catalogos'!$T$2:$T$3</definedName>
+    <definedName name="Parroquia18">'Catalogos'!$U$2:$U$2</definedName>
+    <definedName name="Parroquia19">'Catalogos'!$V$2:$V$3</definedName>
+    <definedName name="Parroquia20">'Catalogos'!$W$2:$W$3</definedName>
+    <definedName name="Parroquia21">'Catalogos'!$X$2:$X$2</definedName>
+    <definedName name="Parroquia22">'Catalogos'!$Y$2:$Y$4</definedName>
+    <definedName name="Parroquia23">'Catalogos'!$Z$2:$Z$6</definedName>
+    <definedName name="Parroquia24">'Catalogos'!$AA$2:$AA$2</definedName>
+    <definedName name="Parroquia25">'Catalogos'!$AB$2:$AB$2</definedName>
+    <definedName name="Parroquia26">'Catalogos'!$AC$2:$AC$2</definedName>
+    <definedName name="Parroquia27">'Catalogos'!$AD$2:$AD$4</definedName>
+    <definedName name="Parroquia28">'Catalogos'!$AE$2:$AE$2</definedName>
+    <definedName name="Parroquia29">'Catalogos'!$AF$2:$AF$5</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
+    <numFmt numFmtId="165" formatCode="dd-mm-yyyy"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -272,7 +307,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -312,6 +347,9 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -901,7 +939,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="n"/>
+      <c r="A4" s="19" t="n"/>
       <c r="B4" s="12" t="n"/>
       <c r="C4" s="12" t="n"/>
       <c r="D4" s="12" t="n"/>
@@ -932,25 +970,28 @@
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="K2:T2"/>
   </mergeCells>
-  <dataValidations count="6">
-    <dataValidation sqref="B4:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Estado no válido" error="Selecciona Táchira." promptTitle="Estado" prompt="Selecciona el estado." type="list">
-      <formula1>"Táchira"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C4:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Municipio no válido" error="Selecciona un municipio del catálogo." promptTitle="Municipio" prompt="Selecciona el municipio." type="list">
-      <formula1>"Andrés Bello,Antonio Rómulo Costa,Ayacucho,Bolívar,Cárdenas,Córdoba,Fernández Feo,Francisco de Miranda,García de Hevia,Guásimos,Independencia,Jáuregui,José María Vargas,Junín,Libertad,Libertador,Lobatera,Michelena,Panamericano,Pedro María Ureña,Rafael Urdaneta,Samuel Darío Maldonado,San Cristóbal,San Judas Tadeo,Seboruco,Simón Rodríguez,Sucre,Torbes,Uribante"</formula1>
-    </dataValidation>
-    <dataValidation sqref="A4:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Fecha no válida" error="Introduce una fecha válida." promptTitle="Fecha" prompt="Selecciona o introduce una fecha." type="date" operator="between">
+  <dataValidations count="7">
+    <dataValidation sqref="A4:A1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Fecha no válida" error="Introduce una fecha válida." promptTitle="" prompt="DD-MM-AAAA" type="date" operator="between">
       <formula1>DATE(1900,1,1)</formula1>
       <formula2>DATE(2100,12,31)</formula2>
     </dataValidation>
-    <dataValidation sqref="I4:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Actividad no válida" error="Selecciona una actividad del catálogo." promptTitle="Actividad desarrollada" prompt="Selecciona el tipo de actividad." type="list">
-      <formula1>"Salud toca tu puerta,Sesiones educativas,Los Comités de Salud van a la escuela,Actividades de Promoción y Prevención Social,Participación Activa en Jornadas,Participación Activa en Inmunizaciones,Entrevista servicio social"</formula1>
+    <dataValidation sqref="B4:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Táchira"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="ASIC no válido" error="Selecciona un ASIC del catálogo." promptTitle="ASIC" prompt="Selecciona el ASIC." type="list">
-      <formula1>"Andrés Bello,Antonio Rómulo Costa,Ayacucho,Bolívar,Capacho Independencia,Capacho Libertad,Cárdenas,Córdoba,Dr. Hugo Murzi,Dr. Jacinto Convit,Dr. José María Vargas,Fernández Feo,García de Hevia,Guásimos,Jáuregui,Junín,Libertador,Michelena,Panamericano,Sabaneta,Samuel Darío Maldonado,Sucre,Torbes,Ureña,Uribante"</formula1>
+    <dataValidation sqref="C4:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Municipio no válido" error="Selecciona un municipio del catálogo." type="list">
+      <formula1>CatalogoMunicipios</formula1>
     </dataValidation>
-    <dataValidation sqref="F4:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Entrada inválida" error="Seleccione un tipo de establecimiento válido" promptTitle="Establecimiento de Salud" prompt="Seleccione el tipo de establecimiento de salud" type="list">
+    <dataValidation sqref="D4:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Parroquia no válida" error="Selecciona una parroquia correspondiente al municipio." type="list">
+      <formula1>INDIRECT("Parroquia"&amp;MATCH(C4,CatalogoMunicipios,0))</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ASIC no válido" error="Selecciona un ASIC del catálogo." type="list">
+      <formula1>CatalogoASIC</formula1>
+    </dataValidation>
+    <dataValidation sqref="F4:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Entrada inválida" error="Seleccione un tipo de establecimiento válido" type="list">
       <formula1>"Consultorio Popular TIPO I,Consultorio Popular TIPO II,Consultorio Popular TIPO III,Clinica Popular TIPO I,Clinica Popular TIPO II,CDI,SRI,CAT,Hospitales TIPO I,Hospitales TIPO II,Hospitales TIPO III,Hospitales TIPO IV"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I4:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Actividad no válida" error="Selecciona una actividad del catálogo." type="list">
+      <formula1>CatalogoActividades</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -958,4 +999,878 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AF30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>CatalogoActividades</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>CatalogoASIC</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>CatalogoMunicipios</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Andrés Bello</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Antonio Rómulo Costa</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Ayacucho</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Cárdenas</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Fernández Feo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Francisco de Miranda</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>García de Hevia</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Guásimos</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Independencia</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>José María Vargas</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Junín</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Jáuregui</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Libertad</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Libertador</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Lobatera</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Michelena</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Panamericano</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Pedro María Ureña</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Rafael Urdaneta</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Samuel Darío Maldonado</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>San Cristóbal</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>San Judas Tadeo</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Seboruco</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>Simón Rodríguez</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>Torbes</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>Uribante</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Actividades de Promoción y Prevención Social</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Andrés Bello</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Andrés Bello</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Cordero</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Virgen del Carmen</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Rivas Berti</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Isaías Medina Angarita</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Amenodoro Rangel Lamús</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Santa Ana del Táchira</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Alberto Adriani</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>San José de Bolívar</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Boca de Grita</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Palmira</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Capacho Nuevo</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>El Cobre</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Bramón</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Emilio Constantino Guerrero</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Capacho Viejo</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Abejales</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Constitución</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Michelena</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>La Palmita</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Nueva Arcadia</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Delicias</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Boconó</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Francisco Romero Lobo</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>San Judas Tadeo</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Seboruco</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>San Simón</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Eleazar López Contreras</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>San Josecito</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Cárdenas</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Entrevista servicio social</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Antonio Rómulo Costa</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Antonio Rómulo Costa</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>San Juan de Colón</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Juan Vicente Gómez</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>La Florida</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>San Rafael del Piñal</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>José Antonio Páez</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Juan Germán Roscio</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>La Petrólea</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>La Grita</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Cipriano Castro</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Doradas</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Lobatera</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>San Pablo</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Ureña</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Hernández</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>La Concordia</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>San Pablo</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>Juan Pablo Peñaloza</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Los Comités de Salud van a la escuela</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ayacucho</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ayacucho</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>San Pedro del Río</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Palotal</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Táriba</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Santo Domingo</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>La Fría</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Román Cárdenas</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Quinimarí</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Monseñor Miguel Antonio Salas</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Manuel Felipe Rugeles</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Emeterio Ochoa</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>La Tendida</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Pedro María Morantes</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Potosí</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Otra nueva</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>San Antonio del Táchira</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Rubio</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>San Joaquín de Navay</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>San Juan Bautista</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>Pregonero</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Participación Activa en Inmunizaciones</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Capacho Independencia</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Cárdenas</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>San Sebastián</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Participación Activa en Jornadas</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Capacho Libertad</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Salud toca tu puerta</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Cárdenas</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Fernández Feo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sesiones educativas</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Francisco de Miranda</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Dr. Hugo Murzi</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>García de Hevia</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Dr. Jacinto Convit</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Guásimos</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Dr. José María Vargas</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Independencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Fernández Feo</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>José María Vargas</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>García de Hevia</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Junín</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Guásimos</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Jáuregui</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Junín</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Libertad</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Jáuregui</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Libertador</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Libertador</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Lobatera</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Michelena</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Michelena</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Panamericano</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Panamericano</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Sabaneta</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Pedro María Ureña</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Samuel Darío Maldonado</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Rafael Urdaneta</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Samuel Darío Maldonado</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Torbes</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>San Cristóbal</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Ureña</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>San Judas Tadeo</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Uribante</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Seboruco</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Simón Rodríguez</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Sucre</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Torbes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Uribante</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>